<commit_message>
edim-ai-blueprint: Task 관련 문서 4종에 작업자 열 추가
- WBS(담당역할과 분리)·기능정의서(178기능)·산출물목록(35종)·RTM(자동 전파)
- 배정은 각 스크립트 ASSIGNEES dict(ID→실명)에 기입 후 재생성 — 기본 '미정'
- RTM은 기능정의서 작업자를 읽어 자동 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/04_WBS/EDIM_WBS.xlsx
+++ b/edim-ai-blueprint/docs/04_WBS/EDIM_WBS.xlsx
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA39"/>
+  <dimension ref="A1:BB39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -732,9 +732,9 @@
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="4" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="2.4" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="2.4" customWidth="1" min="11" max="11"/>
     <col width="2.4" customWidth="1" min="12" max="12"/>
     <col width="2.4" customWidth="1" min="13" max="13"/>
@@ -778,6 +778,7 @@
     <col width="2.4" customWidth="1" min="51" max="51"/>
     <col width="2.4" customWidth="1" min="52" max="52"/>
     <col width="2.4" customWidth="1" min="53" max="53"/>
+    <col width="2.4" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,235 +814,240 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>담당</t>
+          <t>담당(역할)</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
+          <t>작업자</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
           <t>산출물</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>W1</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>W2</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>W3</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>W4</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
         <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>W8</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>W10</t>
         </is>
       </c>
-      <c r="T1" s="5" t="inlineStr">
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="U1" s="5" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="V1" s="5" t="inlineStr">
+      <c r="W1" s="5" t="inlineStr">
         <is>
           <t>W13</t>
         </is>
       </c>
-      <c r="W1" s="5" t="inlineStr">
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>W14</t>
         </is>
       </c>
-      <c r="X1" s="5" t="inlineStr">
+      <c r="Y1" s="5" t="inlineStr">
         <is>
           <t>W15</t>
         </is>
       </c>
-      <c r="Y1" s="5" t="inlineStr">
+      <c r="Z1" s="5" t="inlineStr">
         <is>
           <t>W16</t>
         </is>
       </c>
-      <c r="Z1" s="5" t="inlineStr">
+      <c r="AA1" s="5" t="inlineStr">
         <is>
           <t>W17</t>
         </is>
       </c>
-      <c r="AA1" s="5" t="inlineStr">
+      <c r="AB1" s="5" t="inlineStr">
         <is>
           <t>W18</t>
         </is>
       </c>
-      <c r="AB1" s="5" t="inlineStr">
+      <c r="AC1" s="5" t="inlineStr">
         <is>
           <t>W19</t>
         </is>
       </c>
-      <c r="AC1" s="5" t="inlineStr">
+      <c r="AD1" s="5" t="inlineStr">
         <is>
           <t>W20</t>
         </is>
       </c>
-      <c r="AD1" s="5" t="inlineStr">
+      <c r="AE1" s="5" t="inlineStr">
         <is>
           <t>W21</t>
         </is>
       </c>
-      <c r="AE1" s="5" t="inlineStr">
+      <c r="AF1" s="5" t="inlineStr">
         <is>
           <t>W22</t>
         </is>
       </c>
-      <c r="AF1" s="5" t="inlineStr">
+      <c r="AG1" s="5" t="inlineStr">
         <is>
           <t>W23</t>
         </is>
       </c>
-      <c r="AG1" s="5" t="inlineStr">
+      <c r="AH1" s="5" t="inlineStr">
         <is>
           <t>W24</t>
         </is>
       </c>
-      <c r="AH1" s="5" t="inlineStr">
+      <c r="AI1" s="5" t="inlineStr">
         <is>
           <t>W25</t>
         </is>
       </c>
-      <c r="AI1" s="5" t="inlineStr">
+      <c r="AJ1" s="5" t="inlineStr">
         <is>
           <t>W26</t>
         </is>
       </c>
-      <c r="AJ1" s="5" t="inlineStr">
+      <c r="AK1" s="5" t="inlineStr">
         <is>
           <t>W27</t>
         </is>
       </c>
-      <c r="AK1" s="5" t="inlineStr">
+      <c r="AL1" s="5" t="inlineStr">
         <is>
           <t>W28</t>
         </is>
       </c>
-      <c r="AL1" s="5" t="inlineStr">
+      <c r="AM1" s="5" t="inlineStr">
         <is>
           <t>W29</t>
         </is>
       </c>
-      <c r="AM1" s="5" t="inlineStr">
+      <c r="AN1" s="5" t="inlineStr">
         <is>
           <t>W30</t>
         </is>
       </c>
-      <c r="AN1" s="5" t="inlineStr">
+      <c r="AO1" s="5" t="inlineStr">
         <is>
           <t>W31</t>
         </is>
       </c>
-      <c r="AO1" s="5" t="inlineStr">
+      <c r="AP1" s="5" t="inlineStr">
         <is>
           <t>W32</t>
         </is>
       </c>
-      <c r="AP1" s="5" t="inlineStr">
+      <c r="AQ1" s="5" t="inlineStr">
         <is>
           <t>W33</t>
         </is>
       </c>
-      <c r="AQ1" s="5" t="inlineStr">
+      <c r="AR1" s="5" t="inlineStr">
         <is>
           <t>W34</t>
         </is>
       </c>
-      <c r="AR1" s="5" t="inlineStr">
+      <c r="AS1" s="5" t="inlineStr">
         <is>
           <t>W35</t>
         </is>
       </c>
-      <c r="AS1" s="5" t="inlineStr">
+      <c r="AT1" s="5" t="inlineStr">
         <is>
           <t>W36</t>
         </is>
       </c>
-      <c r="AT1" s="5" t="inlineStr">
+      <c r="AU1" s="5" t="inlineStr">
         <is>
           <t>W37</t>
         </is>
       </c>
-      <c r="AU1" s="5" t="inlineStr">
+      <c r="AV1" s="5" t="inlineStr">
         <is>
           <t>W38</t>
         </is>
       </c>
-      <c r="AV1" s="5" t="inlineStr">
+      <c r="AW1" s="5" t="inlineStr">
         <is>
           <t>W39</t>
         </is>
       </c>
-      <c r="AW1" s="5" t="inlineStr">
+      <c r="AX1" s="5" t="inlineStr">
         <is>
           <t>W40</t>
         </is>
       </c>
-      <c r="AX1" s="5" t="inlineStr">
+      <c r="AY1" s="5" t="inlineStr">
         <is>
           <t>W41</t>
         </is>
       </c>
-      <c r="AY1" s="5" t="inlineStr">
+      <c r="AZ1" s="5" t="inlineStr">
         <is>
           <t>W42</t>
         </is>
       </c>
-      <c r="AZ1" s="5" t="inlineStr">
+      <c r="BA1" s="5" t="inlineStr">
         <is>
           <t>W43</t>
         </is>
       </c>
-      <c r="BA1" s="5" t="inlineStr">
+      <c r="BB1" s="5" t="inlineStr">
         <is>
           <t>W44</t>
         </is>
@@ -1077,11 +1083,11 @@
         <v>2</v>
       </c>
       <c r="G2" s="7" t="inlineStr"/>
-      <c r="H2" s="7" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="7" t="inlineStr"/>
-      <c r="J2" s="8" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr"/>
       <c r="K2" s="8" t="inlineStr"/>
-      <c r="L2" s="9" t="inlineStr"/>
+      <c r="L2" s="8" t="inlineStr"/>
       <c r="M2" s="9" t="inlineStr"/>
       <c r="N2" s="9" t="inlineStr"/>
       <c r="O2" s="9" t="inlineStr"/>
@@ -1123,6 +1129,7 @@
       <c r="AY2" s="9" t="inlineStr"/>
       <c r="AZ2" s="9" t="inlineStr"/>
       <c r="BA2" s="9" t="inlineStr"/>
+      <c r="BB2" s="9" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -1158,14 +1165,18 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>사업수행계획서</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr"/>
-      <c r="J3" s="8" t="inlineStr"/>
-      <c r="K3" s="9" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
+      <c r="K3" s="8" t="inlineStr"/>
       <c r="L3" s="9" t="inlineStr"/>
       <c r="M3" s="9" t="inlineStr"/>
       <c r="N3" s="9" t="inlineStr"/>
@@ -1208,6 +1219,7 @@
       <c r="AY3" s="9" t="inlineStr"/>
       <c r="AZ3" s="9" t="inlineStr"/>
       <c r="BA3" s="9" t="inlineStr"/>
+      <c r="BB3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -1243,19 +1255,23 @@
           <t>인프라</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Jenkins 파이프라인</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>서버·Docker·PG·MinIO 선구축 완료</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr"/>
       <c r="K4" s="8" t="inlineStr"/>
-      <c r="L4" s="9" t="inlineStr"/>
+      <c r="L4" s="8" t="inlineStr"/>
       <c r="M4" s="9" t="inlineStr"/>
       <c r="N4" s="9" t="inlineStr"/>
       <c r="O4" s="9" t="inlineStr"/>
@@ -1297,6 +1313,7 @@
       <c r="AY4" s="9" t="inlineStr"/>
       <c r="AZ4" s="9" t="inlineStr"/>
       <c r="BA4" s="9" t="inlineStr"/>
+      <c r="BB4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -1332,19 +1349,23 @@
           <t>아키텍트</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>개발표준정의서 v1.0</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>백엔드 언어 확정 포함</t>
         </is>
       </c>
-      <c r="J5" s="9" t="inlineStr"/>
-      <c r="K5" s="8" t="inlineStr"/>
-      <c r="L5" s="9" t="inlineStr"/>
+      <c r="K5" s="9" t="inlineStr"/>
+      <c r="L5" s="8" t="inlineStr"/>
       <c r="M5" s="9" t="inlineStr"/>
       <c r="N5" s="9" t="inlineStr"/>
       <c r="O5" s="9" t="inlineStr"/>
@@ -1386,6 +1407,7 @@
       <c r="AY5" s="9" t="inlineStr"/>
       <c r="AZ5" s="9" t="inlineStr"/>
       <c r="BA5" s="9" t="inlineStr"/>
+      <c r="BB5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -1417,15 +1439,15 @@
         <v>4</v>
       </c>
       <c r="G6" s="13" t="inlineStr"/>
-      <c r="H6" s="13" t="inlineStr"/>
+      <c r="H6" s="12" t="inlineStr"/>
       <c r="I6" s="13" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
+      <c r="J6" s="13" t="inlineStr"/>
       <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="14" t="inlineStr"/>
+      <c r="L6" s="9" t="inlineStr"/>
       <c r="M6" s="14" t="inlineStr"/>
       <c r="N6" s="14" t="inlineStr"/>
       <c r="O6" s="14" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
+      <c r="P6" s="14" t="inlineStr"/>
       <c r="Q6" s="9" t="inlineStr"/>
       <c r="R6" s="9" t="inlineStr"/>
       <c r="S6" s="9" t="inlineStr"/>
@@ -1463,6 +1485,7 @@
       <c r="AY6" s="9" t="inlineStr"/>
       <c r="AZ6" s="9" t="inlineStr"/>
       <c r="BA6" s="9" t="inlineStr"/>
+      <c r="BB6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -1498,21 +1521,25 @@
           <t>컨설턴트</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>현행분석서</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>고객사 인터뷰</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="14" t="inlineStr"/>
+      <c r="L7" s="9" t="inlineStr"/>
       <c r="M7" s="14" t="inlineStr"/>
-      <c r="N7" s="9" t="inlineStr"/>
+      <c r="N7" s="14" t="inlineStr"/>
       <c r="O7" s="9" t="inlineStr"/>
       <c r="P7" s="9" t="inlineStr"/>
       <c r="Q7" s="9" t="inlineStr"/>
@@ -1552,6 +1579,7 @@
       <c r="AY7" s="9" t="inlineStr"/>
       <c r="AZ7" s="9" t="inlineStr"/>
       <c r="BA7" s="9" t="inlineStr"/>
+      <c r="BB7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1587,22 +1615,26 @@
           <t>PM·전 파트</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>요구사항정의서 v1.0</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>보안솔루션·DUCT·ERP경계·CAD명령표</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="14" t="inlineStr"/>
+      <c r="L8" s="9" t="inlineStr"/>
       <c r="M8" s="14" t="inlineStr"/>
       <c r="N8" s="14" t="inlineStr"/>
-      <c r="O8" s="9" t="inlineStr"/>
+      <c r="O8" s="14" t="inlineStr"/>
       <c r="P8" s="9" t="inlineStr"/>
       <c r="Q8" s="9" t="inlineStr"/>
       <c r="R8" s="9" t="inlineStr"/>
@@ -1641,6 +1673,7 @@
       <c r="AY8" s="9" t="inlineStr"/>
       <c r="AZ8" s="9" t="inlineStr"/>
       <c r="BA8" s="9" t="inlineStr"/>
+      <c r="BB8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -1676,23 +1709,27 @@
           <t>DBA·AI</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>데이터 이행 계획서 초안</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>AI 학습(RAW DB) 연계</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="9" t="inlineStr"/>
       <c r="L9" s="9" t="inlineStr"/>
       <c r="M9" s="9" t="inlineStr"/>
-      <c r="N9" s="14" t="inlineStr"/>
+      <c r="N9" s="9" t="inlineStr"/>
       <c r="O9" s="14" t="inlineStr"/>
-      <c r="P9" s="9" t="inlineStr"/>
+      <c r="P9" s="14" t="inlineStr"/>
       <c r="Q9" s="9" t="inlineStr"/>
       <c r="R9" s="9" t="inlineStr"/>
       <c r="S9" s="9" t="inlineStr"/>
@@ -1730,6 +1767,7 @@
       <c r="AY9" s="9" t="inlineStr"/>
       <c r="AZ9" s="9" t="inlineStr"/>
       <c r="BA9" s="9" t="inlineStr"/>
+      <c r="BB9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -1765,23 +1803,27 @@
           <t>전체</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
         <is>
           <t>검토회의록</t>
         </is>
       </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>M1: 요구 확정</t>
         </is>
       </c>
-      <c r="J10" s="9" t="inlineStr"/>
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr"/>
       <c r="N10" s="9" t="inlineStr"/>
-      <c r="O10" s="14" t="inlineStr"/>
-      <c r="P10" s="9" t="inlineStr"/>
+      <c r="O10" s="9" t="inlineStr"/>
+      <c r="P10" s="14" t="inlineStr"/>
       <c r="Q10" s="9" t="inlineStr"/>
       <c r="R10" s="9" t="inlineStr"/>
       <c r="S10" s="9" t="inlineStr"/>
@@ -1819,6 +1861,7 @@
       <c r="AY10" s="9" t="inlineStr"/>
       <c r="AZ10" s="9" t="inlineStr"/>
       <c r="BA10" s="9" t="inlineStr"/>
+      <c r="BB10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
@@ -1850,21 +1893,21 @@
         <v>6</v>
       </c>
       <c r="G11" s="16" t="inlineStr"/>
-      <c r="H11" s="16" t="inlineStr"/>
+      <c r="H11" s="15" t="inlineStr"/>
       <c r="I11" s="16" t="inlineStr"/>
-      <c r="J11" s="9" t="inlineStr"/>
+      <c r="J11" s="16" t="inlineStr"/>
       <c r="K11" s="9" t="inlineStr"/>
       <c r="L11" s="9" t="inlineStr"/>
       <c r="M11" s="9" t="inlineStr"/>
       <c r="N11" s="9" t="inlineStr"/>
       <c r="O11" s="9" t="inlineStr"/>
-      <c r="P11" s="17" t="inlineStr"/>
+      <c r="P11" s="9" t="inlineStr"/>
       <c r="Q11" s="17" t="inlineStr"/>
       <c r="R11" s="17" t="inlineStr"/>
       <c r="S11" s="17" t="inlineStr"/>
       <c r="T11" s="17" t="inlineStr"/>
       <c r="U11" s="17" t="inlineStr"/>
-      <c r="V11" s="9" t="inlineStr"/>
+      <c r="V11" s="17" t="inlineStr"/>
       <c r="W11" s="9" t="inlineStr"/>
       <c r="X11" s="9" t="inlineStr"/>
       <c r="Y11" s="9" t="inlineStr"/>
@@ -1896,6 +1939,7 @@
       <c r="AY11" s="9" t="inlineStr"/>
       <c r="AZ11" s="9" t="inlineStr"/>
       <c r="BA11" s="9" t="inlineStr"/>
+      <c r="BB11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1931,23 +1975,27 @@
           <t>UI/UX</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>화면설계서 v1.0</t>
         </is>
       </c>
-      <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="9" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr"/>
       <c r="N12" s="9" t="inlineStr"/>
       <c r="O12" s="9" t="inlineStr"/>
-      <c r="P12" s="17" t="inlineStr"/>
+      <c r="P12" s="9" t="inlineStr"/>
       <c r="Q12" s="17" t="inlineStr"/>
       <c r="R12" s="17" t="inlineStr"/>
       <c r="S12" s="17" t="inlineStr"/>
-      <c r="T12" s="9" t="inlineStr"/>
+      <c r="T12" s="17" t="inlineStr"/>
       <c r="U12" s="9" t="inlineStr"/>
       <c r="V12" s="9" t="inlineStr"/>
       <c r="W12" s="9" t="inlineStr"/>
@@ -1981,6 +2029,7 @@
       <c r="AY12" s="9" t="inlineStr"/>
       <c r="AZ12" s="9" t="inlineStr"/>
       <c r="BA12" s="9" t="inlineStr"/>
+      <c r="BB12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -2016,25 +2065,29 @@
           <t>DBA</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
         <is>
           <t>DB정의서 v1.0 + 마이그레이션</t>
         </is>
       </c>
-      <c r="I13" s="11" t="inlineStr">
+      <c r="J13" s="11" t="inlineStr">
         <is>
           <t>DDL v0.4.1 기반</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="9" t="inlineStr"/>
       <c r="L13" s="9" t="inlineStr"/>
       <c r="M13" s="9" t="inlineStr"/>
       <c r="N13" s="9" t="inlineStr"/>
       <c r="O13" s="9" t="inlineStr"/>
-      <c r="P13" s="17" t="inlineStr"/>
+      <c r="P13" s="9" t="inlineStr"/>
       <c r="Q13" s="17" t="inlineStr"/>
-      <c r="R13" s="9" t="inlineStr"/>
+      <c r="R13" s="17" t="inlineStr"/>
       <c r="S13" s="9" t="inlineStr"/>
       <c r="T13" s="9" t="inlineStr"/>
       <c r="U13" s="9" t="inlineStr"/>
@@ -2070,6 +2123,7 @@
       <c r="AY13" s="9" t="inlineStr"/>
       <c r="AZ13" s="9" t="inlineStr"/>
       <c r="BA13" s="9" t="inlineStr"/>
+      <c r="BB13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -2105,23 +2159,27 @@
           <t>백엔드</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>인터페이스정의서</t>
         </is>
       </c>
-      <c r="I14" s="11" t="inlineStr"/>
-      <c r="J14" s="9" t="inlineStr"/>
+      <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="9" t="inlineStr"/>
       <c r="L14" s="9" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr"/>
       <c r="N14" s="9" t="inlineStr"/>
       <c r="O14" s="9" t="inlineStr"/>
       <c r="P14" s="9" t="inlineStr"/>
-      <c r="Q14" s="17" t="inlineStr"/>
+      <c r="Q14" s="9" t="inlineStr"/>
       <c r="R14" s="17" t="inlineStr"/>
       <c r="S14" s="17" t="inlineStr"/>
-      <c r="T14" s="9" t="inlineStr"/>
+      <c r="T14" s="17" t="inlineStr"/>
       <c r="U14" s="9" t="inlineStr"/>
       <c r="V14" s="9" t="inlineStr"/>
       <c r="W14" s="9" t="inlineStr"/>
@@ -2155,6 +2213,7 @@
       <c r="AY14" s="9" t="inlineStr"/>
       <c r="AZ14" s="9" t="inlineStr"/>
       <c r="BA14" s="9" t="inlineStr"/>
+      <c r="BB14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -2190,13 +2249,17 @@
           <t>아키텍트</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
         <is>
           <t>클래스정의서</t>
         </is>
       </c>
-      <c r="I15" s="11" t="inlineStr"/>
-      <c r="J15" s="9" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
       <c r="K15" s="9" t="inlineStr"/>
       <c r="L15" s="9" t="inlineStr"/>
       <c r="M15" s="9" t="inlineStr"/>
@@ -2204,10 +2267,10 @@
       <c r="O15" s="9" t="inlineStr"/>
       <c r="P15" s="9" t="inlineStr"/>
       <c r="Q15" s="9" t="inlineStr"/>
-      <c r="R15" s="17" t="inlineStr"/>
+      <c r="R15" s="9" t="inlineStr"/>
       <c r="S15" s="17" t="inlineStr"/>
       <c r="T15" s="17" t="inlineStr"/>
-      <c r="U15" s="9" t="inlineStr"/>
+      <c r="U15" s="17" t="inlineStr"/>
       <c r="V15" s="9" t="inlineStr"/>
       <c r="W15" s="9" t="inlineStr"/>
       <c r="X15" s="9" t="inlineStr"/>
@@ -2240,6 +2303,7 @@
       <c r="AY15" s="9" t="inlineStr"/>
       <c r="AZ15" s="9" t="inlineStr"/>
       <c r="BA15" s="9" t="inlineStr"/>
+      <c r="BB15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -2275,17 +2339,21 @@
           <t>전체</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
         <is>
           <t>검토회의록</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="J16" s="11" t="inlineStr">
         <is>
           <t>M2: 설계 완료</t>
         </is>
       </c>
-      <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="9" t="inlineStr"/>
       <c r="L16" s="9" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr"/>
@@ -2296,8 +2364,8 @@
       <c r="R16" s="9" t="inlineStr"/>
       <c r="S16" s="9" t="inlineStr"/>
       <c r="T16" s="9" t="inlineStr"/>
-      <c r="U16" s="17" t="inlineStr"/>
-      <c r="V16" s="9" t="inlineStr"/>
+      <c r="U16" s="9" t="inlineStr"/>
+      <c r="V16" s="17" t="inlineStr"/>
       <c r="W16" s="9" t="inlineStr"/>
       <c r="X16" s="9" t="inlineStr"/>
       <c r="Y16" s="9" t="inlineStr"/>
@@ -2329,6 +2397,7 @@
       <c r="AY16" s="9" t="inlineStr"/>
       <c r="AZ16" s="9" t="inlineStr"/>
       <c r="BA16" s="9" t="inlineStr"/>
+      <c r="BB16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -2360,13 +2429,13 @@
         <v>28</v>
       </c>
       <c r="G17" s="19" t="inlineStr"/>
-      <c r="H17" s="19" t="inlineStr"/>
-      <c r="I17" s="19" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr"/>
+      <c r="I17" s="19" t="inlineStr"/>
+      <c r="J17" s="19" t="inlineStr">
         <is>
           <t>Phase 중첩 진행</t>
         </is>
       </c>
-      <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="9" t="inlineStr"/>
       <c r="L17" s="9" t="inlineStr"/>
       <c r="M17" s="9" t="inlineStr"/>
@@ -2374,7 +2443,7 @@
       <c r="O17" s="9" t="inlineStr"/>
       <c r="P17" s="9" t="inlineStr"/>
       <c r="Q17" s="9" t="inlineStr"/>
-      <c r="R17" s="20" t="inlineStr"/>
+      <c r="R17" s="9" t="inlineStr"/>
       <c r="S17" s="20" t="inlineStr"/>
       <c r="T17" s="20" t="inlineStr"/>
       <c r="U17" s="20" t="inlineStr"/>
@@ -2402,7 +2471,7 @@
       <c r="AQ17" s="20" t="inlineStr"/>
       <c r="AR17" s="20" t="inlineStr"/>
       <c r="AS17" s="20" t="inlineStr"/>
-      <c r="AT17" s="9" t="inlineStr"/>
+      <c r="AT17" s="20" t="inlineStr"/>
       <c r="AU17" s="9" t="inlineStr"/>
       <c r="AV17" s="9" t="inlineStr"/>
       <c r="AW17" s="9" t="inlineStr"/>
@@ -2410,6 +2479,7 @@
       <c r="AY17" s="9" t="inlineStr"/>
       <c r="AZ17" s="9" t="inlineStr"/>
       <c r="BA17" s="9" t="inlineStr"/>
+      <c r="BB17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2445,17 +2515,21 @@
           <t>백엔드 2·FE 1</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>P1 모듈+단위테스트</t>
         </is>
       </c>
-      <c r="I18" s="11" t="inlineStr">
+      <c r="J18" s="11" t="inlineStr">
         <is>
           <t>BOM 전개·Running Test</t>
         </is>
       </c>
-      <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="9" t="inlineStr"/>
       <c r="L18" s="9" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr"/>
@@ -2463,13 +2537,13 @@
       <c r="O18" s="9" t="inlineStr"/>
       <c r="P18" s="9" t="inlineStr"/>
       <c r="Q18" s="9" t="inlineStr"/>
-      <c r="R18" s="20" t="inlineStr"/>
+      <c r="R18" s="9" t="inlineStr"/>
       <c r="S18" s="20" t="inlineStr"/>
       <c r="T18" s="20" t="inlineStr"/>
       <c r="U18" s="20" t="inlineStr"/>
       <c r="V18" s="20" t="inlineStr"/>
       <c r="W18" s="20" t="inlineStr"/>
-      <c r="X18" s="9" t="inlineStr"/>
+      <c r="X18" s="20" t="inlineStr"/>
       <c r="Y18" s="9" t="inlineStr"/>
       <c r="Z18" s="9" t="inlineStr"/>
       <c r="AA18" s="9" t="inlineStr"/>
@@ -2499,6 +2573,7 @@
       <c r="AY18" s="9" t="inlineStr"/>
       <c r="AZ18" s="9" t="inlineStr"/>
       <c r="BA18" s="9" t="inlineStr"/>
+      <c r="BB18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -2534,17 +2609,21 @@
           <t>백엔드 2·FE 2</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr">
         <is>
           <t>P2 모듈</t>
         </is>
       </c>
-      <c r="I19" s="11" t="inlineStr">
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>◆M3(W20): 코드→Run→견적 E2E 데모</t>
         </is>
       </c>
-      <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr"/>
       <c r="M19" s="9" t="inlineStr"/>
@@ -2556,7 +2635,7 @@
       <c r="S19" s="9" t="inlineStr"/>
       <c r="T19" s="9" t="inlineStr"/>
       <c r="U19" s="9" t="inlineStr"/>
-      <c r="V19" s="20" t="inlineStr"/>
+      <c r="V19" s="9" t="inlineStr"/>
       <c r="W19" s="20" t="inlineStr"/>
       <c r="X19" s="20" t="inlineStr"/>
       <c r="Y19" s="20" t="inlineStr"/>
@@ -2564,7 +2643,7 @@
       <c r="AA19" s="20" t="inlineStr"/>
       <c r="AB19" s="20" t="inlineStr"/>
       <c r="AC19" s="20" t="inlineStr"/>
-      <c r="AD19" s="9" t="inlineStr"/>
+      <c r="AD19" s="20" t="inlineStr"/>
       <c r="AE19" s="9" t="inlineStr"/>
       <c r="AF19" s="9" t="inlineStr"/>
       <c r="AG19" s="9" t="inlineStr"/>
@@ -2588,6 +2667,7 @@
       <c r="AY19" s="9" t="inlineStr"/>
       <c r="AZ19" s="9" t="inlineStr"/>
       <c r="BA19" s="9" t="inlineStr"/>
+      <c r="BB19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2623,13 +2703,17 @@
           <t>백엔드 2·FE 1</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
         <is>
           <t>P3 모듈</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr"/>
-      <c r="J20" s="9" t="inlineStr"/>
+      <c r="J20" s="11" t="inlineStr"/>
       <c r="K20" s="9" t="inlineStr"/>
       <c r="L20" s="9" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr"/>
@@ -2647,13 +2731,13 @@
       <c r="Y20" s="9" t="inlineStr"/>
       <c r="Z20" s="9" t="inlineStr"/>
       <c r="AA20" s="9" t="inlineStr"/>
-      <c r="AB20" s="20" t="inlineStr"/>
+      <c r="AB20" s="9" t="inlineStr"/>
       <c r="AC20" s="20" t="inlineStr"/>
       <c r="AD20" s="20" t="inlineStr"/>
       <c r="AE20" s="20" t="inlineStr"/>
       <c r="AF20" s="20" t="inlineStr"/>
       <c r="AG20" s="20" t="inlineStr"/>
-      <c r="AH20" s="9" t="inlineStr"/>
+      <c r="AH20" s="20" t="inlineStr"/>
       <c r="AI20" s="9" t="inlineStr"/>
       <c r="AJ20" s="9" t="inlineStr"/>
       <c r="AK20" s="9" t="inlineStr"/>
@@ -2673,6 +2757,7 @@
       <c r="AY20" s="9" t="inlineStr"/>
       <c r="AZ20" s="9" t="inlineStr"/>
       <c r="BA20" s="9" t="inlineStr"/>
+      <c r="BB20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -2708,17 +2793,21 @@
           <t>백엔드 1·FE 2·AI 1</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>P4 모듈</t>
         </is>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>AI 승인 게이트 포함</t>
         </is>
       </c>
-      <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="9" t="inlineStr"/>
       <c r="L21" s="9" t="inlineStr"/>
       <c r="M21" s="9" t="inlineStr"/>
@@ -2740,7 +2829,7 @@
       <c r="AC21" s="9" t="inlineStr"/>
       <c r="AD21" s="9" t="inlineStr"/>
       <c r="AE21" s="9" t="inlineStr"/>
-      <c r="AF21" s="20" t="inlineStr"/>
+      <c r="AF21" s="9" t="inlineStr"/>
       <c r="AG21" s="20" t="inlineStr"/>
       <c r="AH21" s="20" t="inlineStr"/>
       <c r="AI21" s="20" t="inlineStr"/>
@@ -2748,7 +2837,7 @@
       <c r="AK21" s="20" t="inlineStr"/>
       <c r="AL21" s="20" t="inlineStr"/>
       <c r="AM21" s="20" t="inlineStr"/>
-      <c r="AN21" s="9" t="inlineStr"/>
+      <c r="AN21" s="20" t="inlineStr"/>
       <c r="AO21" s="9" t="inlineStr"/>
       <c r="AP21" s="9" t="inlineStr"/>
       <c r="AQ21" s="9" t="inlineStr"/>
@@ -2762,6 +2851,7 @@
       <c r="AY21" s="9" t="inlineStr"/>
       <c r="AZ21" s="9" t="inlineStr"/>
       <c r="BA21" s="9" t="inlineStr"/>
+      <c r="BB21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -2797,13 +2887,17 @@
           <t>백엔드 2·FE 1·모바일 1</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
         <is>
           <t>P5 모듈</t>
         </is>
       </c>
-      <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="9" t="inlineStr"/>
+      <c r="J22" s="11" t="inlineStr"/>
       <c r="K22" s="9" t="inlineStr"/>
       <c r="L22" s="9" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr"/>
@@ -2829,7 +2923,7 @@
       <c r="AG22" s="9" t="inlineStr"/>
       <c r="AH22" s="9" t="inlineStr"/>
       <c r="AI22" s="9" t="inlineStr"/>
-      <c r="AJ22" s="20" t="inlineStr"/>
+      <c r="AJ22" s="9" t="inlineStr"/>
       <c r="AK22" s="20" t="inlineStr"/>
       <c r="AL22" s="20" t="inlineStr"/>
       <c r="AM22" s="20" t="inlineStr"/>
@@ -2839,7 +2933,7 @@
       <c r="AQ22" s="20" t="inlineStr"/>
       <c r="AR22" s="20" t="inlineStr"/>
       <c r="AS22" s="20" t="inlineStr"/>
-      <c r="AT22" s="9" t="inlineStr"/>
+      <c r="AT22" s="20" t="inlineStr"/>
       <c r="AU22" s="9" t="inlineStr"/>
       <c r="AV22" s="9" t="inlineStr"/>
       <c r="AW22" s="9" t="inlineStr"/>
@@ -2847,6 +2941,7 @@
       <c r="AY22" s="9" t="inlineStr"/>
       <c r="AZ22" s="9" t="inlineStr"/>
       <c r="BA22" s="9" t="inlineStr"/>
+      <c r="BB22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -2882,17 +2977,21 @@
           <t>전 개발</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>단위테스트 결과</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>개발표준 §7</t>
         </is>
       </c>
-      <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="9" t="inlineStr"/>
       <c r="L23" s="9" t="inlineStr"/>
       <c r="M23" s="9" t="inlineStr"/>
@@ -2900,7 +2999,7 @@
       <c r="O23" s="9" t="inlineStr"/>
       <c r="P23" s="9" t="inlineStr"/>
       <c r="Q23" s="9" t="inlineStr"/>
-      <c r="R23" s="20" t="inlineStr"/>
+      <c r="R23" s="9" t="inlineStr"/>
       <c r="S23" s="20" t="inlineStr"/>
       <c r="T23" s="20" t="inlineStr"/>
       <c r="U23" s="20" t="inlineStr"/>
@@ -2928,7 +3027,7 @@
       <c r="AQ23" s="20" t="inlineStr"/>
       <c r="AR23" s="20" t="inlineStr"/>
       <c r="AS23" s="20" t="inlineStr"/>
-      <c r="AT23" s="9" t="inlineStr"/>
+      <c r="AT23" s="20" t="inlineStr"/>
       <c r="AU23" s="9" t="inlineStr"/>
       <c r="AV23" s="9" t="inlineStr"/>
       <c r="AW23" s="9" t="inlineStr"/>
@@ -2936,6 +3035,7 @@
       <c r="AY23" s="9" t="inlineStr"/>
       <c r="AZ23" s="9" t="inlineStr"/>
       <c r="BA23" s="9" t="inlineStr"/>
+      <c r="BB23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
@@ -2967,9 +3067,9 @@
         <v>8</v>
       </c>
       <c r="G24" s="22" t="inlineStr"/>
-      <c r="H24" s="22" t="inlineStr"/>
+      <c r="H24" s="21" t="inlineStr"/>
       <c r="I24" s="22" t="inlineStr"/>
-      <c r="J24" s="9" t="inlineStr"/>
+      <c r="J24" s="22" t="inlineStr"/>
       <c r="K24" s="9" t="inlineStr"/>
       <c r="L24" s="9" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr"/>
@@ -2999,7 +3099,7 @@
       <c r="AK24" s="9" t="inlineStr"/>
       <c r="AL24" s="9" t="inlineStr"/>
       <c r="AM24" s="9" t="inlineStr"/>
-      <c r="AN24" s="23" t="inlineStr"/>
+      <c r="AN24" s="9" t="inlineStr"/>
       <c r="AO24" s="23" t="inlineStr"/>
       <c r="AP24" s="23" t="inlineStr"/>
       <c r="AQ24" s="23" t="inlineStr"/>
@@ -3007,12 +3107,13 @@
       <c r="AS24" s="23" t="inlineStr"/>
       <c r="AT24" s="23" t="inlineStr"/>
       <c r="AU24" s="23" t="inlineStr"/>
-      <c r="AV24" s="9" t="inlineStr"/>
+      <c r="AV24" s="23" t="inlineStr"/>
       <c r="AW24" s="9" t="inlineStr"/>
       <c r="AX24" s="9" t="inlineStr"/>
       <c r="AY24" s="9" t="inlineStr"/>
       <c r="AZ24" s="9" t="inlineStr"/>
       <c r="BA24" s="9" t="inlineStr"/>
+      <c r="BB24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -3048,17 +3149,21 @@
           <t>QA·전 파트</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>통합테스트 결과</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>개요 §7 워크플로우 기반</t>
         </is>
       </c>
-      <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="9" t="inlineStr"/>
       <c r="L25" s="9" t="inlineStr"/>
       <c r="M25" s="9" t="inlineStr"/>
@@ -3088,13 +3193,13 @@
       <c r="AK25" s="9" t="inlineStr"/>
       <c r="AL25" s="9" t="inlineStr"/>
       <c r="AM25" s="9" t="inlineStr"/>
-      <c r="AN25" s="23" t="inlineStr"/>
+      <c r="AN25" s="9" t="inlineStr"/>
       <c r="AO25" s="23" t="inlineStr"/>
       <c r="AP25" s="23" t="inlineStr"/>
       <c r="AQ25" s="23" t="inlineStr"/>
       <c r="AR25" s="23" t="inlineStr"/>
       <c r="AS25" s="23" t="inlineStr"/>
-      <c r="AT25" s="9" t="inlineStr"/>
+      <c r="AT25" s="23" t="inlineStr"/>
       <c r="AU25" s="9" t="inlineStr"/>
       <c r="AV25" s="9" t="inlineStr"/>
       <c r="AW25" s="9" t="inlineStr"/>
@@ -3102,6 +3207,7 @@
       <c r="AY25" s="9" t="inlineStr"/>
       <c r="AZ25" s="9" t="inlineStr"/>
       <c r="BA25" s="9" t="inlineStr"/>
+      <c r="BB25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -3137,17 +3243,21 @@
           <t>QA·인프라</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>성능시험 결과</t>
         </is>
       </c>
-      <c r="I26" s="11" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>산출물 1시간·BOM 30초·응답 2/3초</t>
         </is>
       </c>
-      <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="9" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr"/>
@@ -3181,16 +3291,17 @@
       <c r="AO26" s="9" t="inlineStr"/>
       <c r="AP26" s="9" t="inlineStr"/>
       <c r="AQ26" s="9" t="inlineStr"/>
-      <c r="AR26" s="23" t="inlineStr"/>
+      <c r="AR26" s="9" t="inlineStr"/>
       <c r="AS26" s="23" t="inlineStr"/>
       <c r="AT26" s="23" t="inlineStr"/>
-      <c r="AU26" s="9" t="inlineStr"/>
+      <c r="AU26" s="23" t="inlineStr"/>
       <c r="AV26" s="9" t="inlineStr"/>
       <c r="AW26" s="9" t="inlineStr"/>
       <c r="AX26" s="9" t="inlineStr"/>
       <c r="AY26" s="9" t="inlineStr"/>
       <c r="AZ26" s="9" t="inlineStr"/>
       <c r="BA26" s="9" t="inlineStr"/>
+      <c r="BB26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -3226,13 +3337,17 @@
           <t>전 개발</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
         <is>
           <t>결함관리대장</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr"/>
-      <c r="J27" s="9" t="inlineStr"/>
+      <c r="J27" s="11" t="inlineStr"/>
       <c r="K27" s="9" t="inlineStr"/>
       <c r="L27" s="9" t="inlineStr"/>
       <c r="M27" s="9" t="inlineStr"/>
@@ -3264,18 +3379,19 @@
       <c r="AM27" s="9" t="inlineStr"/>
       <c r="AN27" s="9" t="inlineStr"/>
       <c r="AO27" s="9" t="inlineStr"/>
-      <c r="AP27" s="23" t="inlineStr"/>
+      <c r="AP27" s="9" t="inlineStr"/>
       <c r="AQ27" s="23" t="inlineStr"/>
       <c r="AR27" s="23" t="inlineStr"/>
       <c r="AS27" s="23" t="inlineStr"/>
       <c r="AT27" s="23" t="inlineStr"/>
       <c r="AU27" s="23" t="inlineStr"/>
-      <c r="AV27" s="9" t="inlineStr"/>
+      <c r="AV27" s="23" t="inlineStr"/>
       <c r="AW27" s="9" t="inlineStr"/>
       <c r="AX27" s="9" t="inlineStr"/>
       <c r="AY27" s="9" t="inlineStr"/>
       <c r="AZ27" s="9" t="inlineStr"/>
       <c r="BA27" s="9" t="inlineStr"/>
+      <c r="BB27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -3311,13 +3427,17 @@
           <t>QA·PM</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
         <is>
           <t>기능확인서 초안</t>
         </is>
       </c>
-      <c r="I28" s="11" t="inlineStr"/>
-      <c r="J28" s="9" t="inlineStr"/>
+      <c r="J28" s="11" t="inlineStr"/>
       <c r="K28" s="9" t="inlineStr"/>
       <c r="L28" s="9" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr"/>
@@ -3353,14 +3473,15 @@
       <c r="AQ28" s="9" t="inlineStr"/>
       <c r="AR28" s="9" t="inlineStr"/>
       <c r="AS28" s="9" t="inlineStr"/>
-      <c r="AT28" s="23" t="inlineStr"/>
+      <c r="AT28" s="9" t="inlineStr"/>
       <c r="AU28" s="23" t="inlineStr"/>
-      <c r="AV28" s="9" t="inlineStr"/>
+      <c r="AV28" s="23" t="inlineStr"/>
       <c r="AW28" s="9" t="inlineStr"/>
       <c r="AX28" s="9" t="inlineStr"/>
       <c r="AY28" s="9" t="inlineStr"/>
       <c r="AZ28" s="9" t="inlineStr"/>
       <c r="BA28" s="9" t="inlineStr"/>
+      <c r="BB28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
@@ -3392,9 +3513,9 @@
         <v>6</v>
       </c>
       <c r="G29" s="25" t="inlineStr"/>
-      <c r="H29" s="25" t="inlineStr"/>
+      <c r="H29" s="24" t="inlineStr"/>
       <c r="I29" s="25" t="inlineStr"/>
-      <c r="J29" s="9" t="inlineStr"/>
+      <c r="J29" s="25" t="inlineStr"/>
       <c r="K29" s="9" t="inlineStr"/>
       <c r="L29" s="9" t="inlineStr"/>
       <c r="M29" s="9" t="inlineStr"/>
@@ -3428,16 +3549,17 @@
       <c r="AO29" s="9" t="inlineStr"/>
       <c r="AP29" s="9" t="inlineStr"/>
       <c r="AQ29" s="9" t="inlineStr"/>
-      <c r="AR29" s="26" t="inlineStr"/>
+      <c r="AR29" s="9" t="inlineStr"/>
       <c r="AS29" s="26" t="inlineStr"/>
       <c r="AT29" s="26" t="inlineStr"/>
       <c r="AU29" s="26" t="inlineStr"/>
       <c r="AV29" s="26" t="inlineStr"/>
       <c r="AW29" s="26" t="inlineStr"/>
-      <c r="AX29" s="9" t="inlineStr"/>
+      <c r="AX29" s="26" t="inlineStr"/>
       <c r="AY29" s="9" t="inlineStr"/>
       <c r="AZ29" s="9" t="inlineStr"/>
       <c r="BA29" s="9" t="inlineStr"/>
+      <c r="BB29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -3473,17 +3595,21 @@
           <t>DBA·컨설턴트</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>이행 결과서</t>
         </is>
       </c>
-      <c r="I30" s="11" t="inlineStr">
+      <c r="J30" s="11" t="inlineStr">
         <is>
           <t>★검증 필수</t>
         </is>
       </c>
-      <c r="J30" s="9" t="inlineStr"/>
       <c r="K30" s="9" t="inlineStr"/>
       <c r="L30" s="9" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr"/>
@@ -3517,16 +3643,17 @@
       <c r="AO30" s="9" t="inlineStr"/>
       <c r="AP30" s="9" t="inlineStr"/>
       <c r="AQ30" s="9" t="inlineStr"/>
-      <c r="AR30" s="26" t="inlineStr"/>
+      <c r="AR30" s="9" t="inlineStr"/>
       <c r="AS30" s="26" t="inlineStr"/>
       <c r="AT30" s="26" t="inlineStr"/>
       <c r="AU30" s="26" t="inlineStr"/>
-      <c r="AV30" s="9" t="inlineStr"/>
+      <c r="AV30" s="26" t="inlineStr"/>
       <c r="AW30" s="9" t="inlineStr"/>
       <c r="AX30" s="9" t="inlineStr"/>
       <c r="AY30" s="9" t="inlineStr"/>
       <c r="AZ30" s="9" t="inlineStr"/>
       <c r="BA30" s="9" t="inlineStr"/>
+      <c r="BB30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -3562,17 +3689,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
         <is>
           <t>학습 DB·품질 리포트</t>
         </is>
       </c>
-      <c r="I31" s="11" t="inlineStr">
+      <c r="J31" s="11" t="inlineStr">
         <is>
           <t>슬라이드 25 파이프라인</t>
         </is>
       </c>
-      <c r="J31" s="9" t="inlineStr"/>
       <c r="K31" s="9" t="inlineStr"/>
       <c r="L31" s="9" t="inlineStr"/>
       <c r="M31" s="9" t="inlineStr"/>
@@ -3608,14 +3739,15 @@
       <c r="AQ31" s="9" t="inlineStr"/>
       <c r="AR31" s="9" t="inlineStr"/>
       <c r="AS31" s="9" t="inlineStr"/>
-      <c r="AT31" s="26" t="inlineStr"/>
+      <c r="AT31" s="9" t="inlineStr"/>
       <c r="AU31" s="26" t="inlineStr"/>
       <c r="AV31" s="26" t="inlineStr"/>
       <c r="AW31" s="26" t="inlineStr"/>
-      <c r="AX31" s="9" t="inlineStr"/>
+      <c r="AX31" s="26" t="inlineStr"/>
       <c r="AY31" s="9" t="inlineStr"/>
       <c r="AZ31" s="9" t="inlineStr"/>
       <c r="BA31" s="9" t="inlineStr"/>
+      <c r="BB31" s="9" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -3651,17 +3783,21 @@
           <t>인프라</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
         <is>
           <t>설치·배포 매뉴얼</t>
         </is>
       </c>
-      <c r="I32" s="11" t="inlineStr">
+      <c r="J32" s="11" t="inlineStr">
         <is>
           <t>Self-managed 대응</t>
         </is>
       </c>
-      <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="9" t="inlineStr"/>
       <c r="L32" s="9" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr"/>
@@ -3698,13 +3834,14 @@
       <c r="AR32" s="9" t="inlineStr"/>
       <c r="AS32" s="9" t="inlineStr"/>
       <c r="AT32" s="9" t="inlineStr"/>
-      <c r="AU32" s="26" t="inlineStr"/>
+      <c r="AU32" s="9" t="inlineStr"/>
       <c r="AV32" s="26" t="inlineStr"/>
       <c r="AW32" s="26" t="inlineStr"/>
-      <c r="AX32" s="9" t="inlineStr"/>
+      <c r="AX32" s="26" t="inlineStr"/>
       <c r="AY32" s="9" t="inlineStr"/>
       <c r="AZ32" s="9" t="inlineStr"/>
       <c r="BA32" s="9" t="inlineStr"/>
+      <c r="BB32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
@@ -3736,9 +3873,9 @@
         <v>4</v>
       </c>
       <c r="G33" s="28" t="inlineStr"/>
-      <c r="H33" s="28" t="inlineStr"/>
+      <c r="H33" s="27" t="inlineStr"/>
       <c r="I33" s="28" t="inlineStr"/>
-      <c r="J33" s="9" t="inlineStr"/>
+      <c r="J33" s="28" t="inlineStr"/>
       <c r="K33" s="9" t="inlineStr"/>
       <c r="L33" s="9" t="inlineStr"/>
       <c r="M33" s="9" t="inlineStr"/>
@@ -3776,12 +3913,13 @@
       <c r="AS33" s="9" t="inlineStr"/>
       <c r="AT33" s="9" t="inlineStr"/>
       <c r="AU33" s="9" t="inlineStr"/>
-      <c r="AV33" s="29" t="inlineStr"/>
+      <c r="AV33" s="9" t="inlineStr"/>
       <c r="AW33" s="29" t="inlineStr"/>
       <c r="AX33" s="29" t="inlineStr"/>
       <c r="AY33" s="29" t="inlineStr"/>
-      <c r="AZ33" s="9" t="inlineStr"/>
+      <c r="AZ33" s="29" t="inlineStr"/>
       <c r="BA33" s="9" t="inlineStr"/>
+      <c r="BB33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -3817,13 +3955,17 @@
           <t>전체</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr">
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
         <is>
           <t>운영 리포트</t>
         </is>
       </c>
-      <c r="I34" s="11" t="inlineStr"/>
-      <c r="J34" s="9" t="inlineStr"/>
+      <c r="J34" s="11" t="inlineStr"/>
       <c r="K34" s="9" t="inlineStr"/>
       <c r="L34" s="9" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr"/>
@@ -3861,12 +4003,13 @@
       <c r="AS34" s="9" t="inlineStr"/>
       <c r="AT34" s="9" t="inlineStr"/>
       <c r="AU34" s="9" t="inlineStr"/>
-      <c r="AV34" s="29" t="inlineStr"/>
+      <c r="AV34" s="9" t="inlineStr"/>
       <c r="AW34" s="29" t="inlineStr"/>
       <c r="AX34" s="29" t="inlineStr"/>
       <c r="AY34" s="29" t="inlineStr"/>
-      <c r="AZ34" s="9" t="inlineStr"/>
+      <c r="AZ34" s="29" t="inlineStr"/>
       <c r="BA34" s="9" t="inlineStr"/>
+      <c r="BB34" s="9" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -3902,13 +4045,17 @@
           <t>PM·컨설턴트</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
         <is>
           <t>교육 자료·결과</t>
         </is>
       </c>
-      <c r="I35" s="11" t="inlineStr"/>
-      <c r="J35" s="9" t="inlineStr"/>
+      <c r="J35" s="11" t="inlineStr"/>
       <c r="K35" s="9" t="inlineStr"/>
       <c r="L35" s="9" t="inlineStr"/>
       <c r="M35" s="9" t="inlineStr"/>
@@ -3947,11 +4094,12 @@
       <c r="AT35" s="9" t="inlineStr"/>
       <c r="AU35" s="9" t="inlineStr"/>
       <c r="AV35" s="9" t="inlineStr"/>
-      <c r="AW35" s="29" t="inlineStr"/>
+      <c r="AW35" s="9" t="inlineStr"/>
       <c r="AX35" s="29" t="inlineStr"/>
-      <c r="AY35" s="9" t="inlineStr"/>
+      <c r="AY35" s="29" t="inlineStr"/>
       <c r="AZ35" s="9" t="inlineStr"/>
       <c r="BA35" s="9" t="inlineStr"/>
+      <c r="BB35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -3987,13 +4135,17 @@
           <t>테크니컬라이터</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr">
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
         <is>
           <t>매뉴얼 2종</t>
         </is>
       </c>
-      <c r="I36" s="11" t="inlineStr"/>
-      <c r="J36" s="9" t="inlineStr"/>
+      <c r="J36" s="11" t="inlineStr"/>
       <c r="K36" s="9" t="inlineStr"/>
       <c r="L36" s="9" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr"/>
@@ -4031,12 +4183,13 @@
       <c r="AS36" s="9" t="inlineStr"/>
       <c r="AT36" s="9" t="inlineStr"/>
       <c r="AU36" s="9" t="inlineStr"/>
-      <c r="AV36" s="29" t="inlineStr"/>
+      <c r="AV36" s="9" t="inlineStr"/>
       <c r="AW36" s="29" t="inlineStr"/>
       <c r="AX36" s="29" t="inlineStr"/>
-      <c r="AY36" s="9" t="inlineStr"/>
+      <c r="AY36" s="29" t="inlineStr"/>
       <c r="AZ36" s="9" t="inlineStr"/>
       <c r="BA36" s="9" t="inlineStr"/>
+      <c r="BB36" s="9" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="30" t="inlineStr">
@@ -4068,9 +4221,9 @@
         <v>2</v>
       </c>
       <c r="G37" s="31" t="inlineStr"/>
-      <c r="H37" s="31" t="inlineStr"/>
+      <c r="H37" s="30" t="inlineStr"/>
       <c r="I37" s="31" t="inlineStr"/>
-      <c r="J37" s="9" t="inlineStr"/>
+      <c r="J37" s="31" t="inlineStr"/>
       <c r="K37" s="9" t="inlineStr"/>
       <c r="L37" s="9" t="inlineStr"/>
       <c r="M37" s="9" t="inlineStr"/>
@@ -4112,8 +4265,9 @@
       <c r="AW37" s="9" t="inlineStr"/>
       <c r="AX37" s="9" t="inlineStr"/>
       <c r="AY37" s="9" t="inlineStr"/>
-      <c r="AZ37" s="32" t="inlineStr"/>
+      <c r="AZ37" s="9" t="inlineStr"/>
       <c r="BA37" s="32" t="inlineStr"/>
+      <c r="BB37" s="32" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -4149,17 +4303,21 @@
           <t>고객·PM</t>
         </is>
       </c>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
         <is>
           <t>기능확인서 승인</t>
         </is>
       </c>
-      <c r="I38" s="11" t="inlineStr">
+      <c r="J38" s="11" t="inlineStr">
         <is>
           <t>M4: 검수</t>
         </is>
       </c>
-      <c r="J38" s="9" t="inlineStr"/>
       <c r="K38" s="9" t="inlineStr"/>
       <c r="L38" s="9" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr"/>
@@ -4201,8 +4359,9 @@
       <c r="AW38" s="9" t="inlineStr"/>
       <c r="AX38" s="9" t="inlineStr"/>
       <c r="AY38" s="9" t="inlineStr"/>
-      <c r="AZ38" s="32" t="inlineStr"/>
-      <c r="BA38" s="9" t="inlineStr"/>
+      <c r="AZ38" s="9" t="inlineStr"/>
+      <c r="BA38" s="32" t="inlineStr"/>
+      <c r="BB38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -4238,13 +4397,17 @@
           <t>PM</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr">
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
         <is>
           <t>완료보고서</t>
         </is>
       </c>
-      <c r="I39" s="11" t="inlineStr"/>
-      <c r="J39" s="9" t="inlineStr"/>
+      <c r="J39" s="11" t="inlineStr"/>
       <c r="K39" s="9" t="inlineStr"/>
       <c r="L39" s="9" t="inlineStr"/>
       <c r="M39" s="9" t="inlineStr"/>
@@ -4287,7 +4450,8 @@
       <c r="AX39" s="9" t="inlineStr"/>
       <c r="AY39" s="9" t="inlineStr"/>
       <c r="AZ39" s="9" t="inlineStr"/>
-      <c r="BA39" s="32" t="inlineStr"/>
+      <c r="BA39" s="9" t="inlineStr"/>
+      <c r="BB39" s="32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>